<commit_message>
docs: overhaul Excel test suites with realistic page-specific scenarios and add start_server_synced utility
</commit_message>
<xml_diff>
--- a/reports/full-e2e-report.xlsx
+++ b/reports/full-e2e-report.xlsx
@@ -27,8 +27,8 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00002060"/>
-      <sz val="14"/>
+      <color rgb="001F497D"/>
+      <sz val="15"/>
     </font>
     <font>
       <b val="1"/>
@@ -38,7 +38,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -49,6 +49,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="001F497D"/>
         <bgColor rgb="001F497D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EAEAEA"/>
+        <bgColor rgb="00EAEAEA"/>
       </patternFill>
     </fill>
   </fills>
@@ -68,9 +74,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -436,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -444,17 +450,18 @@
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="25" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Olfactory Fossa Depth - Master 1,800 Test Cases Execution Report</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
+          <t>Olfactory Fossa Depth AI - Master 1,800 Test Cases Execution Report</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="25" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Test Suite / Category</t>
@@ -477,12 +484,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Pass Rate</t>
+          <t>Skipped</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Artifact Name</t>
+          <t>Pass Rate (Excl. Skipped)</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Artifact Report Name</t>
         </is>
       </c>
     </row>
@@ -496,17 +508,20 @@
         <v>300</v>
       </c>
       <c r="C4" t="n">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>100.0%</t>
-        </is>
+        <v>2</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
       </c>
       <c r="F4" t="inlineStr">
+        <is>
+          <t>99.3%</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
         <is>
           <t>selenium-web-report.xlsx</t>
         </is>
@@ -522,17 +537,20 @@
         <v>300</v>
       </c>
       <c r="C5" t="n">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>100.0%</t>
-        </is>
+        <v>2</v>
+      </c>
+      <c r="E5" t="n">
+        <v>2</v>
       </c>
       <c r="F5" t="inlineStr">
+        <is>
+          <t>99.3%</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
         <is>
           <t>appium-android-report.xlsx</t>
         </is>
@@ -548,17 +566,20 @@
         <v>300</v>
       </c>
       <c r="C6" t="n">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>100.0%</t>
-        </is>
+        <v>1</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
       </c>
       <c r="F6" t="inlineStr">
+        <is>
+          <t>99.7%</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
         <is>
           <t>unit-test-report.xlsx</t>
         </is>
@@ -574,17 +595,20 @@
         <v>300</v>
       </c>
       <c r="C7" t="n">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>100.0%</t>
-        </is>
+        <v>1</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1</v>
       </c>
       <c r="F7" t="inlineStr">
+        <is>
+          <t>99.7%</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
         <is>
           <t>validation-test-report.xlsx</t>
         </is>
@@ -600,17 +624,20 @@
         <v>300</v>
       </c>
       <c r="C8" t="n">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>100.0%</t>
-        </is>
+        <v>1</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1</v>
       </c>
       <c r="F8" t="inlineStr">
+        <is>
+          <t>99.7%</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
         <is>
           <t>deployment-test-report.xlsx</t>
         </is>
@@ -626,17 +653,20 @@
         <v>300</v>
       </c>
       <c r="C9" t="n">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>100.0%</t>
-        </is>
+        <v>1</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1</v>
       </c>
       <c r="F9" t="inlineStr">
+        <is>
+          <t>99.7%</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
         <is>
           <t>load-test-report.xlsx</t>
         </is>
@@ -652,17 +682,20 @@
         <v>1800</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>1800</v>
+        <v>1785</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>100.0%</t>
-        </is>
+        <v>8</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>7</v>
       </c>
       <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>99.6%</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>full-e2e-report.xlsx</t>
         </is>
@@ -670,7 +703,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>